<commit_message>
Add About and Members pages; move editorial histories into Resources
- Add about.html (mission, principles, interim steering group, policies)
- Add members.html (people directory from editorial_histories.xlsx, CC BY-NC CSV export)
- Add assets/ui.js (license-gate modal + dataset download helpers)
- Convert editors.html to a redirect into resources.html#editorial-histories
- Rework resources.html into Reading/Editorial-histories tabs
- Unify nav across all pages: Home · About · Journals · Integrity · Resources · Join
- Update data sources and indexing/editorial spreadsheets; refresh README

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/xlsx/editorial_histories.xlsx
+++ b/data/xlsx/editorial_histories.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G213"/>
+  <dimension ref="A1:H216"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -540,6 +540,11 @@
           <t>Source</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -577,6 +582,11 @@
           <t>McCarthy ISME history; College Music Symposium</t>
         </is>
       </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>In memoriam (2001)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -614,6 +624,11 @@
           <t>IJME Cumulative Index Nos. 1-6 (archive.org)</t>
         </is>
       </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>In memoriam (2003)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -651,6 +666,7 @@
           <t>Internet Archive (controlled-lending issues)</t>
         </is>
       </c>
+      <c r="H4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -688,6 +704,11 @@
           <t>IJME Cumulative Index Nos. 25-30 (archive.org)</t>
         </is>
       </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>In memoriam (2008)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -725,6 +746,7 @@
           <t>IJME Cumulative Index Nos. 25-30 (archive.org)</t>
         </is>
       </c>
+      <c r="H6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -762,6 +784,7 @@
           <t>IJME indexes 2004-06; Ilari &amp; Johnson 26(1) 2008</t>
         </is>
       </c>
+      <c r="H7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -799,6 +822,7 @@
           <t>IJME index 2004 (Practice 22(3))</t>
         </is>
       </c>
+      <c r="H8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -836,6 +860,7 @@
           <t>IJME index 2004, 22(3)</t>
         </is>
       </c>
+      <c r="H9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -873,6 +898,7 @@
           <t>IJME indexes 2005 (23(3)), 2006 (24(3))</t>
         </is>
       </c>
+      <c r="H10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -910,6 +936,7 @@
           <t>Editorials 26(1) 2008, 27(1) 2009, 28(3) 2010</t>
         </is>
       </c>
+      <c r="H11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -947,6 +974,7 @@
           <t>ISME McPherson bio; Vol 28(3) 2010</t>
         </is>
       </c>
+      <c r="H12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -984,6 +1012,7 @@
           <t>36(1) 2018 editorial; 31(1) 2013</t>
         </is>
       </c>
+      <c r="H13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1021,6 +1050,7 @@
           <t>36(1) 2018 editorial; EdUHK profile</t>
         </is>
       </c>
+      <c r="H14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1058,6 +1088,7 @@
           <t>Harrison bio, TEXT Special Issue 22 (Oct 2013)</t>
         </is>
       </c>
+      <c r="H15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1095,6 +1126,7 @@
           <t>34(2) 2016; mastheads Vol 38-39; gone Vol 40</t>
         </is>
       </c>
+      <c r="H16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1132,6 +1164,7 @@
           <t>mastheads Vol 37-42; 43(1) 2025 editorial</t>
         </is>
       </c>
+      <c r="H17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1169,6 +1202,7 @@
           <t>masthead Vol 39(1) 2021 onward</t>
         </is>
       </c>
+      <c r="H18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1206,6 +1240,7 @@
           <t>masthead Vol 42(1) 2024 onward</t>
         </is>
       </c>
+      <c r="H19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1243,6 +1278,7 @@
           <t>masthead Vol 43(1) 2025; 2025 editorial</t>
         </is>
       </c>
+      <c r="H20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1280,6 +1316,7 @@
           <t>thefreelibrary.com IJME masthead; ISME publications</t>
         </is>
       </c>
+      <c r="H21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1317,6 +1354,7 @@
           <t>journals.sagepub.com/editorial-board/RIM</t>
         </is>
       </c>
+      <c r="H22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1354,6 +1392,7 @@
           <t>revistaeducacionmusical.org editorialTeam</t>
         </is>
       </c>
+      <c r="H23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1391,6 +1430,7 @@
           <t>revistaeducacionmusical.org editorialTeam</t>
         </is>
       </c>
+      <c r="H24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1428,6 +1468,7 @@
           <t>revistaeducacionmusical.org editorialTeam</t>
         </is>
       </c>
+      <c r="H25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -1465,6 +1506,7 @@
           <t>tandfonline.com/journals/cmue20</t>
         </is>
       </c>
+      <c r="H26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -1502,6 +1544,7 @@
           <t>rcm.ac.uk research people 05248</t>
         </is>
       </c>
+      <c r="H27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -1539,6 +1582,7 @@
           <t>tandfonline.com 2025 handover editorial</t>
         </is>
       </c>
+      <c r="H28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -1576,6 +1620,7 @@
           <t>tandfonline.com 2025 handover editorial</t>
         </is>
       </c>
+      <c r="H29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -1613,6 +1658,7 @@
           <t>luca-arts.be/nl/thomas-de-baets</t>
         </is>
       </c>
+      <c r="H30" s="4" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -1650,6 +1696,7 @@
           <t>tandfonline.com cmue20 editorial board</t>
         </is>
       </c>
+      <c r="H31" s="4" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -1687,6 +1734,7 @@
           <t>tandfonline.com cmue20 editorial board</t>
         </is>
       </c>
+      <c r="H32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -1724,6 +1772,7 @@
           <t>tandfonline.com cmue20 editorial board</t>
         </is>
       </c>
+      <c r="H33" s="4" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1761,6 +1810,7 @@
           <t>cambridge.org 1998 handover editorial</t>
         </is>
       </c>
+      <c r="H34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1798,6 +1848,7 @@
           <t>cambridge.org 1998 handover editorial</t>
         </is>
       </c>
+      <c r="H35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1835,6 +1886,7 @@
           <t>eric.ed.gov/?id=EJ1073543</t>
         </is>
       </c>
+      <c r="H36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1872,6 +1924,7 @@
           <t>academia.edu/56542725</t>
         </is>
       </c>
+      <c r="H37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1909,6 +1962,7 @@
           <t>academia.edu/56542725</t>
         </is>
       </c>
+      <c r="H38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1946,6 +2000,7 @@
           <t>cambridge.org editorial board</t>
         </is>
       </c>
+      <c r="H39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -1983,6 +2038,7 @@
           <t>music.illinois.edu/people/profiles/richard-colwell</t>
         </is>
       </c>
+      <c r="H40" s="4" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -2020,6 +2076,11 @@
           <t>en.wikipedia.org/wiki/Bulletin_of_the_Council_for_Research_in_Music_Education</t>
         </is>
       </c>
+      <c r="H41" s="4" t="inlineStr">
+        <is>
+          <t>In memoriam (1995)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
@@ -2057,6 +2118,11 @@
           <t>Wikipedia: BCRME</t>
         </is>
       </c>
+      <c r="H42" s="4" t="inlineStr">
+        <is>
+          <t>In memoriam (2009)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -2094,6 +2160,7 @@
           <t>Wikipedia: BCRME</t>
         </is>
       </c>
+      <c r="H43" s="4" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
@@ -2131,6 +2198,7 @@
           <t>Wikipedia: BCRME</t>
         </is>
       </c>
+      <c r="H44" s="4" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -2168,6 +2236,7 @@
           <t>Wikipedia: BCRME</t>
         </is>
       </c>
+      <c r="H45" s="4" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -2205,6 +2274,7 @@
           <t>Wikipedia: BCRME</t>
         </is>
       </c>
+      <c r="H46" s="4" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -2242,6 +2312,7 @@
           <t>music.illinois.edu/people/profiles/janet-revell-barrett</t>
         </is>
       </c>
+      <c r="H47" s="4" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
@@ -2279,6 +2350,7 @@
           <t>press.uillinois.edu CRME co-editors announcement</t>
         </is>
       </c>
+      <c r="H48" s="4" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
@@ -2316,6 +2388,7 @@
           <t>press.uillinois.edu/journals/?id=bcrme</t>
         </is>
       </c>
+      <c r="H49" s="4" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -2353,6 +2426,7 @@
           <t>digitalcommons.lib.uconn.edu/vrme/vol1/iss1</t>
         </is>
       </c>
+      <c r="H50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -2390,6 +2464,7 @@
           <t>digitalcommons.lib.uconn.edu/vrme/vol2/iss1</t>
         </is>
       </c>
+      <c r="H51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -2427,6 +2502,7 @@
           <t>digitalcommons.lib.uconn.edu/vrme/vol38/iss1/1</t>
         </is>
       </c>
+      <c r="H52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -2464,6 +2540,7 @@
           <t>digitalcommons.lib.uconn.edu/vrme/vol39/iss1/1</t>
         </is>
       </c>
+      <c r="H53" s="2" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -2501,6 +2578,7 @@
           <t>digitalcommons.lib.uconn.edu/vrme/vol47/iss1/1</t>
         </is>
       </c>
+      <c r="H54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -2538,6 +2616,7 @@
           <t>digitalcommons.lib.uconn.edu/vrme/editorialboard.html</t>
         </is>
       </c>
+      <c r="H55" s="2" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
@@ -2575,6 +2654,7 @@
           <t>mdpi.com/2304-6775/5/2/13</t>
         </is>
       </c>
+      <c r="H56" s="4" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
@@ -2612,6 +2692,7 @@
           <t>mdpi.com/2304-6775/5/2/13</t>
         </is>
       </c>
+      <c r="H57" s="4" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
@@ -2649,6 +2730,7 @@
           <t>mdpi.com/2304-6775/5/2/13</t>
         </is>
       </c>
+      <c r="H58" s="4" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
@@ -2686,6 +2768,7 @@
           <t>mdpi.com/2304-6775/5/2/13</t>
         </is>
       </c>
+      <c r="H59" s="4" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
@@ -2723,6 +2806,7 @@
           <t>mdpi.com/2304-6775/5/2/13</t>
         </is>
       </c>
+      <c r="H60" s="4" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
@@ -2760,6 +2844,7 @@
           <t>usm.maine.edu Kaschub profile; MEJ editorial 2020 (10.1177/0027432120924443)</t>
         </is>
       </c>
+      <c r="H61" s="4" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
@@ -2797,6 +2882,7 @@
           <t>nafme.org/member-profile/corin-overland</t>
         </is>
       </c>
+      <c r="H62" s="4" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
@@ -2834,6 +2920,7 @@
           <t>MEJ 'From the Academic Editor' 2023 (10.1177/00274321231218871)</t>
         </is>
       </c>
+      <c r="H63" s="4" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
@@ -2871,6 +2958,7 @@
           <t>nafme.org 2026 Call for Nominations MEJ</t>
         </is>
       </c>
+      <c r="H64" s="4" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
@@ -2908,6 +2996,7 @@
           <t>music.msu.edu/faculty/ryan-shaw</t>
         </is>
       </c>
+      <c r="H65" s="4" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -2945,6 +3034,11 @@
           <t>en.wikipedia.org/wiki/Allen_Britton</t>
         </is>
       </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>In memoriam (2003)</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -2982,6 +3076,11 @@
           <t>isme.org/news/vale-james-c-carlsen</t>
         </is>
       </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>In memoriam (2020)</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -3019,6 +3118,11 @@
           <t>Humphreys &amp; Stauffer 2000 JRME 48(1)</t>
         </is>
       </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>In memoriam (2018)</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
@@ -3056,6 +3160,7 @@
           <t>jstor.org/stable/40319354</t>
         </is>
       </c>
+      <c r="H69" s="3" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -3093,6 +3198,11 @@
           <t>journals.sagepub.com/doi/abs/10.1177/002242940605400201</t>
         </is>
       </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>In memoriam (2022)</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -3130,6 +3240,7 @@
           <t>music.missouri.edu/people/sims</t>
         </is>
       </c>
+      <c r="H71" s="2" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -3167,6 +3278,7 @@
           <t>music.washington.edu/news/2015/01/26</t>
         </is>
       </c>
+      <c r="H72" s="2" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -3204,6 +3316,7 @@
           <t>nafme.org/group/jrme-editorial-committee</t>
         </is>
       </c>
+      <c r="H73" s="2" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -3241,6 +3354,7 @@
           <t>nafme.org/group/jrme-editorial-committee</t>
         </is>
       </c>
+      <c r="H74" s="2" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -3278,6 +3392,7 @@
           <t>journals.sagepub.com/editorial-board/jrm</t>
         </is>
       </c>
+      <c r="H75" s="2" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
@@ -3315,6 +3430,7 @@
           <t>User-provided; hartford.edu Hartt faculty</t>
         </is>
       </c>
+      <c r="H76" s="4" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -3352,6 +3468,7 @@
           <t>en.wikipedia.org/wiki/Gary_E._McPherson</t>
         </is>
       </c>
+      <c r="H77" s="2" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -3389,6 +3506,7 @@
           <t>research.monash.edu RSME editorial</t>
         </is>
       </c>
+      <c r="H78" s="2" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -3426,6 +3544,7 @@
           <t>sempre.org.uk/news/201</t>
         </is>
       </c>
+      <c r="H79" s="2" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -3463,6 +3582,7 @@
           <t>journals.sagepub.com/editorial-board/RSM</t>
         </is>
       </c>
+      <c r="H80" s="2" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -3500,6 +3620,7 @@
           <t>journals.sagepub.com/editorial-board/RSM</t>
         </is>
       </c>
+      <c r="H81" s="2" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -3537,6 +3658,7 @@
           <t>journals.sagepub.com/editorial-board/rsm</t>
         </is>
       </c>
+      <c r="H82" s="2" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
@@ -3574,6 +3696,7 @@
           <t>bibliolore.org 2009/10/22</t>
         </is>
       </c>
+      <c r="H83" s="4" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
@@ -3611,6 +3734,7 @@
           <t>intellectbooks.com/international-journal-of-community-music</t>
         </is>
       </c>
+      <c r="H84" s="4" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
@@ -3648,6 +3772,7 @@
           <t>yorksj.ac.uk/iccm professor-lee-higgins</t>
         </is>
       </c>
+      <c r="H85" s="4" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
@@ -3685,6 +3810,7 @@
           <t>intellectbooks.com/international-journal-of-community-music</t>
         </is>
       </c>
+      <c r="H86" s="4" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
@@ -3722,6 +3848,7 @@
           <t>intellectbooks.com IJCM</t>
         </is>
       </c>
+      <c r="H87" s="4" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
@@ -3759,6 +3886,7 @@
           <t>intellectbooks.com IJCM</t>
         </is>
       </c>
+      <c r="H88" s="4" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -3796,6 +3924,7 @@
           <t>Vol.1 Iss.1 (Collins)</t>
         </is>
       </c>
+      <c r="H89" s="2" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -3833,6 +3962,7 @@
           <t>hull.ac.uk/staff-directory/andrew-king</t>
         </is>
       </c>
+      <c r="H90" s="2" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -3870,6 +4000,7 @@
           <t>intellectbooks.com JMTE</t>
         </is>
       </c>
+      <c r="H91" s="2" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -3907,6 +4038,7 @@
           <t>music.uwo.ca/faculty/bios/adam-patrick-bell.html</t>
         </is>
       </c>
+      <c r="H92" s="2" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -3944,6 +4076,7 @@
           <t>ISME profile; Routledge/OUP bios</t>
         </is>
       </c>
+      <c r="H93" s="2" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -3981,6 +4114,7 @@
           <t>intellectbooks.com JMTE</t>
         </is>
       </c>
+      <c r="H94" s="2" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -4018,6 +4152,7 @@
           <t>intellectbooks.com JMTE</t>
         </is>
       </c>
+      <c r="H95" s="2" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -4055,6 +4190,7 @@
           <t>intellectbooks.com JMTE</t>
         </is>
       </c>
+      <c r="H96" s="2" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -4092,6 +4228,7 @@
           <t>intellectbooks.com JMTE</t>
         </is>
       </c>
+      <c r="H97" s="2" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -4129,6 +4266,7 @@
           <t>intellectbooks.com JMTE</t>
         </is>
       </c>
+      <c r="H98" s="2" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -4166,6 +4304,7 @@
           <t>intellectbooks.com JMTE</t>
         </is>
       </c>
+      <c r="H99" s="2" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
@@ -4203,6 +4342,7 @@
           <t>journals.sagepub.com/toc/jmta/20/1</t>
         </is>
       </c>
+      <c r="H100" s="4" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
@@ -4240,6 +4380,7 @@
           <t>smte.us SMTE bibliography</t>
         </is>
       </c>
+      <c r="H101" s="4" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
@@ -4277,6 +4418,7 @@
           <t>smte.us SMTE bibliography</t>
         </is>
       </c>
+      <c r="H102" s="4" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
@@ -4314,6 +4456,7 @@
           <t>smte.us SMTE bibliography</t>
         </is>
       </c>
+      <c r="H103" s="4" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
@@ -4351,6 +4494,7 @@
           <t>journals.sagepub.com/editorial-board/JMT</t>
         </is>
       </c>
+      <c r="H104" s="4" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
@@ -4388,6 +4532,7 @@
           <t>colorado.edu/music/2016/11/17/taking-lead</t>
         </is>
       </c>
+      <c r="H105" s="4" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="4" t="inlineStr">
@@ -4425,6 +4570,7 @@
           <t>nafme.org/group/jmte-editorial-committee</t>
         </is>
       </c>
+      <c r="H106" s="4" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
@@ -4462,6 +4608,7 @@
           <t>journals.sagepub.com/editorial-board/jmt</t>
         </is>
       </c>
+      <c r="H107" s="4" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -4499,6 +4646,7 @@
           <t>journals.sagepub.com/page/pom 40th anniversary</t>
         </is>
       </c>
+      <c r="H108" s="2" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
@@ -4536,6 +4684,7 @@
           <t>SAGE 40th anniversary collection</t>
         </is>
       </c>
+      <c r="H109" s="3" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -4573,6 +4722,7 @@
           <t>SAGE 40th anniversary collection</t>
         </is>
       </c>
+      <c r="H110" s="2" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -4610,6 +4760,7 @@
           <t>SAGE 40th anniversary collection</t>
         </is>
       </c>
+      <c r="H111" s="2" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -4647,6 +4798,7 @@
           <t>SAGE 40th anniversary collection</t>
         </is>
       </c>
+      <c r="H112" s="2" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -4684,6 +4836,7 @@
           <t>SAGE 40th anniversary collection</t>
         </is>
       </c>
+      <c r="H113" s="2" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -4721,6 +4874,7 @@
           <t>raymondmacdonald.co.uk/biography</t>
         </is>
       </c>
+      <c r="H114" s="2" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -4758,6 +4912,7 @@
           <t>journals.sagepub.com/editorial-board/pom</t>
         </is>
       </c>
+      <c r="H115" s="2" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -4795,6 +4950,7 @@
           <t>eca.ed.ac.uk/profile/dr-nikki-moran</t>
         </is>
       </c>
+      <c r="H116" s="2" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -4832,6 +4988,7 @@
           <t>sagepub.com PoM submission guidelines</t>
         </is>
       </c>
+      <c r="H117" s="2" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -4869,6 +5026,7 @@
           <t>journals.sagepub.com/editorial-board/pom</t>
         </is>
       </c>
+      <c r="H118" s="2" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -4906,6 +5064,7 @@
           <t>journals.sagepub.com/editorial-board/pom</t>
         </is>
       </c>
+      <c r="H119" s="2" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="4" t="inlineStr">
@@ -4943,6 +5102,7 @@
           <t>journals.sagepub.com/toc/gmta/1/1</t>
         </is>
       </c>
+      <c r="H120" s="4" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="3" t="inlineStr">
@@ -4980,6 +5140,7 @@
           <t>SAGE archive</t>
         </is>
       </c>
+      <c r="H121" s="3" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="4" t="inlineStr">
@@ -5017,6 +5178,7 @@
           <t>journals.sagepub.com/toc/gmtb/7/1</t>
         </is>
       </c>
+      <c r="H122" s="4" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="3" t="inlineStr">
@@ -5054,6 +5216,7 @@
           <t>SAGE archive</t>
         </is>
       </c>
+      <c r="H123" s="3" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="4" t="inlineStr">
@@ -5091,6 +5254,7 @@
           <t>journals.sagepub.com/toc/gmtb/14/1</t>
         </is>
       </c>
+      <c r="H124" s="4" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="4" t="inlineStr">
@@ -5128,6 +5292,11 @@
           <t>trinity.edu/directory/dpersell</t>
         </is>
       </c>
+      <c r="H125" s="4" t="inlineStr">
+        <is>
+          <t>In memoriam (2024)</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="4" t="inlineStr">
@@ -5165,6 +5334,7 @@
           <t>unomaha.edu faculty Shelly Cooper</t>
         </is>
       </c>
+      <c r="H126" s="4" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="4" t="inlineStr">
@@ -5202,6 +5372,7 @@
           <t>nafme.org rebrand blog JGME</t>
         </is>
       </c>
+      <c r="H127" s="4" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="4" t="inlineStr">
@@ -5239,6 +5410,7 @@
           <t>journals.sagepub.com/doi/10.1177/27527646241283564</t>
         </is>
       </c>
+      <c r="H128" s="4" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -5276,6 +5448,11 @@
           <t>jstor.org/journal/jhistresemusiedu</t>
         </is>
       </c>
+      <c r="H129" s="2" t="inlineStr">
+        <is>
+          <t>In memoriam (2004)</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -5313,6 +5490,7 @@
           <t>search.asu.edu/profile/198/cv</t>
         </is>
       </c>
+      <c r="H130" s="2" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -5350,6 +5528,7 @@
           <t>ithaca.edu/faculty/fonder/editorship</t>
         </is>
       </c>
+      <c r="H131" s="2" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -5387,6 +5566,7 @@
           <t>isme.org/member/marie-mccarthy; smtd.umich.edu 2022 award</t>
         </is>
       </c>
+      <c r="H132" s="2" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -5424,6 +5604,7 @@
           <t>journals.sagepub.com/editorial-board/jhr</t>
         </is>
       </c>
+      <c r="H133" s="2" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -5461,6 +5642,7 @@
           <t>journals.sagepub.com/editorial-board/jhr</t>
         </is>
       </c>
+      <c r="H134" s="2" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="4" t="inlineStr">
@@ -5498,6 +5680,11 @@
           <t>act.maydaygroup.org/about-us</t>
         </is>
       </c>
+      <c r="H135" s="4" t="inlineStr">
+        <is>
+          <t>In memoriam (2024)</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="4" t="inlineStr">
@@ -5535,6 +5722,7 @@
           <t>act.maydaygroup.org/articles/Bowman6_3.pdf</t>
         </is>
       </c>
+      <c r="H136" s="4" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="4" t="inlineStr">
@@ -5572,6 +5760,7 @@
           <t>act.maydaygroup.org/articles/Elliott12_3.pdf</t>
         </is>
       </c>
+      <c r="H137" s="4" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="4" t="inlineStr">
@@ -5609,6 +5798,7 @@
           <t>act.maydaygroup.org/articles/Bates14_1.pdf</t>
         </is>
       </c>
+      <c r="H138" s="4" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
@@ -5646,6 +5836,7 @@
           <t>act.maydaygroup.org/articles/BradleyGoble22_3.pdf</t>
         </is>
       </c>
+      <c r="H139" s="4" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" s="4" t="inlineStr">
@@ -5683,6 +5874,7 @@
           <t>act.maydaygroup.org/contact-information</t>
         </is>
       </c>
+      <c r="H140" s="4" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
@@ -5720,6 +5912,7 @@
           <t>act.maydaygroup.org/editorial-board</t>
         </is>
       </c>
+      <c r="H141" s="4" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" s="4" t="inlineStr">
@@ -5757,6 +5950,7 @@
           <t>act.maydaygroup.org/editorial-board</t>
         </is>
       </c>
+      <c r="H142" s="4" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="4" t="inlineStr">
@@ -5794,6 +5988,7 @@
           <t>act.maydaygroup.org/editorial-board</t>
         </is>
       </c>
+      <c r="H143" s="4" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -5831,6 +6026,7 @@
           <t>iupress.org/journals/pmer</t>
         </is>
       </c>
+      <c r="H144" s="2" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -5868,6 +6064,7 @@
           <t>scholarworks.iu.edu/iupjournals PMER editorial team</t>
         </is>
       </c>
+      <c r="H145" s="2" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -5905,6 +6102,7 @@
           <t>music.indiana.edu news 2025/02</t>
         </is>
       </c>
+      <c r="H146" s="2" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -5942,6 +6140,7 @@
           <t>iupress.org/journals/pmer</t>
         </is>
       </c>
+      <c r="H147" s="2" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -5979,6 +6178,7 @@
           <t>iupress.org/journals/pmer</t>
         </is>
       </c>
+      <c r="H148" s="2" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
@@ -6016,6 +6216,7 @@
           <t>ijea.org/editors.html (Founding Editors)</t>
         </is>
       </c>
+      <c r="H149" s="4" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="4" t="inlineStr">
@@ -6053,6 +6254,7 @@
           <t>ijea.org/editors.html (Founding Editors)</t>
         </is>
       </c>
+      <c r="H150" s="4" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
@@ -6090,6 +6292,7 @@
           <t>ijea.org/editors.html (Past Managing Editors)</t>
         </is>
       </c>
+      <c r="H151" s="4" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" s="4" t="inlineStr">
@@ -6127,6 +6330,7 @@
           <t>ijea.org/editors.html; mastheads v9–v13</t>
         </is>
       </c>
+      <c r="H152" s="4" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
@@ -6164,6 +6368,7 @@
           <t>ijea.org/editors.html (Past Managing Editors)</t>
         </is>
       </c>
+      <c r="H153" s="4" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="4" t="inlineStr">
@@ -6201,6 +6406,7 @@
           <t>ijea.org/editors.html; mastheads v15–v16</t>
         </is>
       </c>
+      <c r="H154" s="4" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="4" t="inlineStr">
@@ -6238,6 +6444,7 @@
           <t>ijea.org/editors.html; mastheads v12–v15</t>
         </is>
       </c>
+      <c r="H155" s="4" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="4" t="inlineStr">
@@ -6275,6 +6482,7 @@
           <t>ijea.org/editors.html; masthead v15n1 2014</t>
         </is>
       </c>
+      <c r="H156" s="4" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
@@ -6312,6 +6520,7 @@
           <t>ijea.org/editors.html; mastheads v15–v23</t>
         </is>
       </c>
+      <c r="H157" s="4" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
@@ -6349,6 +6558,7 @@
           <t>ijea.org/editors.html (Past Managing Editors)</t>
         </is>
       </c>
+      <c r="H158" s="4" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
@@ -6386,6 +6596,11 @@
           <t>ijea.org/editors.html; mastheads v16, v18</t>
         </is>
       </c>
+      <c r="H159" s="4" t="inlineStr">
+        <is>
+          <t>In memoriam (2023)</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="4" t="inlineStr">
@@ -6423,6 +6638,7 @@
           <t>masthead v18n1 2017</t>
         </is>
       </c>
+      <c r="H160" s="4" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
@@ -6460,6 +6676,7 @@
           <t>mastheads v18(2017), v20(2019), v21(2020)</t>
         </is>
       </c>
+      <c r="H161" s="4" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" s="4" t="inlineStr">
@@ -6497,6 +6714,7 @@
           <t>mastheads v20(2019), v21(2020)</t>
         </is>
       </c>
+      <c r="H162" s="4" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
@@ -6534,6 +6752,7 @@
           <t>ijea.org/editors.html; mastheads v20–v22</t>
         </is>
       </c>
+      <c r="H163" s="4" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" s="4" t="inlineStr">
@@ -6571,6 +6790,7 @@
           <t>ijea.org/editors.html; mastheads v22–v23</t>
         </is>
       </c>
+      <c r="H164" s="4" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" s="4" t="inlineStr">
@@ -6608,6 +6828,7 @@
           <t>mastheads v22(2021), v23(2022)</t>
         </is>
       </c>
+      <c r="H165" s="4" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" s="4" t="inlineStr">
@@ -6645,6 +6866,7 @@
           <t>ijea.org/editors.html; mastheads v22–v25</t>
         </is>
       </c>
+      <c r="H166" s="4" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" s="4" t="inlineStr">
@@ -6682,6 +6904,7 @@
           <t>mastheads v21–v25</t>
         </is>
       </c>
+      <c r="H167" s="4" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" s="4" t="inlineStr">
@@ -6719,6 +6942,7 @@
           <t>ijea.org/editors.html; mastheads v24–v25</t>
         </is>
       </c>
+      <c r="H168" s="4" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
@@ -6756,6 +6980,7 @@
           <t>ijea.org/editors.html</t>
         </is>
       </c>
+      <c r="H169" s="4" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" s="4" t="inlineStr">
@@ -6793,6 +7018,7 @@
           <t>ijea.org/editors.html; mastheads v24–v25</t>
         </is>
       </c>
+      <c r="H170" s="4" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" s="4" t="inlineStr">
@@ -6830,6 +7056,7 @@
           <t>ijea.org/editors.html; mastheads v24–v25</t>
         </is>
       </c>
+      <c r="H171" s="4" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" s="4" t="inlineStr">
@@ -6867,6 +7094,7 @@
           <t>ijea.org/editors.html; mastheads v24–v25</t>
         </is>
       </c>
+      <c r="H172" s="4" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" s="4" t="inlineStr">
@@ -6904,6 +7132,7 @@
           <t>ijea.org/editors.html; mastheads v9–v10</t>
         </is>
       </c>
+      <c r="H173" s="4" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" s="4" t="inlineStr">
@@ -6941,6 +7170,7 @@
           <t>journals.psu.edu/ijea/Former_Editors</t>
         </is>
       </c>
+      <c r="H174" s="4" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" s="4" t="inlineStr">
@@ -6978,6 +7208,7 @@
           <t>journals.psu.edu/ijea/Former_Editors</t>
         </is>
       </c>
+      <c r="H175" s="4" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" s="4" t="inlineStr">
@@ -7015,6 +7246,7 @@
           <t>ijea.org mastheads v10-v13</t>
         </is>
       </c>
+      <c r="H176" s="4" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" s="4" t="inlineStr">
@@ -7052,6 +7284,7 @@
           <t>ijea.org/editors.html</t>
         </is>
       </c>
+      <c r="H177" s="4" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
@@ -7089,6 +7322,11 @@
           <t>Rohwer, Legacy of Charles Elliott, Update 2015</t>
         </is>
       </c>
+      <c r="H178" s="2" t="inlineStr">
+        <is>
+          <t>In memoriam</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="3" t="inlineStr">
@@ -7126,6 +7364,7 @@
           <t>Update 33(1) 2014</t>
         </is>
       </c>
+      <c r="H179" s="3" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
@@ -7163,6 +7402,7 @@
           <t>Update editorials 2014-2015</t>
         </is>
       </c>
+      <c r="H180" s="2" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
@@ -7200,6 +7440,7 @@
           <t>journals.sagepub.com/editorial-board/UPD</t>
         </is>
       </c>
+      <c r="H181" s="2" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
@@ -7237,6 +7478,7 @@
           <t>journals.sagepub.com/editorial-board/UPD</t>
         </is>
       </c>
+      <c r="H182" s="2" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
@@ -7274,6 +7516,7 @@
           <t>journals.sagepub.com/editorial-board/upd</t>
         </is>
       </c>
+      <c r="H183" s="2" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" s="4" t="inlineStr">
@@ -7311,6 +7554,7 @@
           <t>acda.org IJRCS editorial board</t>
         </is>
       </c>
+      <c r="H184" s="4" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" s="4" t="inlineStr">
@@ -7348,6 +7592,7 @@
           <t>acda.org IJRCS editorial board</t>
         </is>
       </c>
+      <c r="H185" s="4" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" s="4" t="inlineStr">
@@ -7385,6 +7630,7 @@
           <t>acda.org IJRCS editorial board</t>
         </is>
       </c>
+      <c r="H186" s="4" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" s="4" t="inlineStr">
@@ -7422,6 +7668,7 @@
           <t>acda.org/publications/international-journal-of-research-in-choral-singing/ijrcs-editorial-board</t>
         </is>
       </c>
+      <c r="H187" s="4" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
@@ -7459,6 +7706,7 @@
           <t>acda.org/publications/choral-journal/contact-choral-journal</t>
         </is>
       </c>
+      <c r="H188" s="2" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" s="4" t="inlineStr">
@@ -7496,6 +7744,7 @@
           <t>digitalcollections.lipscomb.edu/jmtp</t>
         </is>
       </c>
+      <c r="H189" s="4" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" s="4" t="inlineStr">
@@ -7533,6 +7782,7 @@
           <t>digitalcollections.lipscomb.edu/jmtp</t>
         </is>
       </c>
+      <c r="H190" s="4" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" s="4" t="inlineStr">
@@ -7570,6 +7820,7 @@
           <t>digitalcollections.lipscomb.edu/jmtp</t>
         </is>
       </c>
+      <c r="H191" s="4" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" s="4" t="inlineStr">
@@ -7607,6 +7858,7 @@
           <t>digitalcollections.lipscomb.edu/jmtp</t>
         </is>
       </c>
+      <c r="H192" s="4" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
@@ -7644,6 +7896,7 @@
           <t>fjme.journal.fi</t>
         </is>
       </c>
+      <c r="H193" s="2" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" s="4" t="inlineStr">
@@ -7681,6 +7934,7 @@
           <t>asme.edu.au/core-activities/ajme</t>
         </is>
       </c>
+      <c r="H194" s="4" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
@@ -7718,6 +7972,7 @@
           <t>nrme.no editorialTeam</t>
         </is>
       </c>
+      <c r="H195" s="2" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" s="4" t="inlineStr">
@@ -7755,6 +8010,7 @@
           <t>cmea.ca/en/call-for-editors-and-book-proposals</t>
         </is>
       </c>
+      <c r="H196" s="4" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
@@ -7792,6 +8048,7 @@
           <t>revistas.ucm.es/index.php/RECI/about/editorialTeam</t>
         </is>
       </c>
+      <c r="H197" s="2" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" s="4" t="inlineStr">
@@ -7829,6 +8086,7 @@
           <t>ojs.uv.es/index.php/LEEME</t>
         </is>
       </c>
+      <c r="H198" s="4" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
@@ -7866,6 +8124,7 @@
           <t>revistaabem.abem.mus.br editorialTeam</t>
         </is>
       </c>
+      <c r="H199" s="2" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" s="4" t="inlineStr">
@@ -7903,6 +8162,7 @@
           <t>revistascientificas.filo.uba.ar/oidopensante</t>
         </is>
       </c>
+      <c r="H200" s="4" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
@@ -7940,6 +8200,7 @@
           <t>eeme.gr</t>
         </is>
       </c>
+      <c r="H201" s="2" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" s="4" t="inlineStr">
@@ -7977,6 +8238,7 @@
           <t>mtnlake.net; Oxford Handbook chapter</t>
         </is>
       </c>
+      <c r="H202" s="4" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
@@ -8014,6 +8276,7 @@
           <t>intellectbooks.com JPME</t>
         </is>
       </c>
+      <c r="H203" s="2" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
@@ -8051,6 +8314,7 @@
           <t>intellectbooks.com JPME</t>
         </is>
       </c>
+      <c r="H204" s="2" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
@@ -8088,6 +8352,7 @@
           <t>intellectbooks.com/journal-of-popular-music-education</t>
         </is>
       </c>
+      <c r="H205" s="2" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
@@ -8125,6 +8390,7 @@
           <t>intellectbooks.com/journal-of-popular-music-education</t>
         </is>
       </c>
+      <c r="H206" s="2" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" s="4" t="inlineStr">
@@ -8162,6 +8428,7 @@
           <t>kjrme.org/sub/about-editorial</t>
         </is>
       </c>
+      <c r="H207" s="4" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
@@ -8199,6 +8466,7 @@
           <t>ejournal.upsi.edu.my/index.php/MJM/about/editorialTeam</t>
         </is>
       </c>
+      <c r="H208" s="2" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
@@ -8236,6 +8504,7 @@
           <t>ejournal.upsi.edu.my/index.php/MJM/about/editorialTeam</t>
         </is>
       </c>
+      <c r="H209" s="2" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" s="4" t="inlineStr">
@@ -8273,6 +8542,7 @@
           <t>jstage.jst.go.jp/browse/jjomep</t>
         </is>
       </c>
+      <c r="H210" s="4" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
@@ -8310,6 +8580,7 @@
           <t>zgyljy.qk580.com</t>
         </is>
       </c>
+      <c r="H211" s="2" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" s="4" t="inlineStr">
@@ -8347,6 +8618,7 @@
           <t>eduhk.hk/cca</t>
         </is>
       </c>
+      <c r="H212" s="4" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
@@ -8384,6 +8656,121 @@
           <t>baike.baidu.com/item/音乐研究; CNKI MUSI</t>
         </is>
       </c>
+      <c r="H213" s="2" t="inlineStr"/>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>Journal of the Association for Technology in Music Instruction (JATMI)</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Barbara Murphy</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Co-editor</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>present</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>University of Tennessee, Knoxville</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>Verified (ATMI editorial board)</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>atmimusic.com/jatmi-editorial-board-2</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr"/>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>Journal of the Association for Technology in Music Instruction (JATMI)</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Mark Lochstampfor</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>Co-editor</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>present</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>Capital University (retired)</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>Verified (ATMI editorial board)</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>atmimusic.com/jatmi-editorial-board-2</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr"/>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>College Music Symposium</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>James A. Grymes</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Editor</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>present</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>University of North Carolina at Charlotte</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>Verified (CMS)</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>symposium.music.org</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H213"/>

</xml_diff>

<commit_message>
Rework Members into Current/Past editor tabs; refresh datasets
- members.html: split into Current Editors (grouped by journal) and Past
  Editors (who's-who) tabs; split multi-name editor cells; retitle to
  "Editors of the Field"; update CSV export
- Refresh editorial_histories.xlsx and journal_indexing.xlsx data

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/xlsx/editorial_histories.xlsx
+++ b/data/xlsx/editorial_histories.xlsx
@@ -1141,7 +1141,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Co-Editor-in-Chief</t>
+          <t>Co-Editor</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1179,7 +1179,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Co-Editor-in-Chief</t>
+          <t>Co-Editor</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Co-Editor-in-Chief</t>
+          <t>Co-Editor</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1255,7 +1255,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Co-Editor-in-Chief</t>
+          <t>Co-Editor</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -2512,7 +2512,7 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Joseph Michael Abramo</t>
+          <t>Joseph Abramo</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Reindex Chinese journals English-first so they sort alphabetically
Chinese journal names now lead with the English translation followed by the
(simplified) characters, e.g. "Music Research (音乐研究)", so they interleave
in alphabetical listings instead of clustering last.

- journals.js: reorder the 7 Chinese titles; clear now-redundant trans
- journal_indexing.xlsx: rewrite 7 "《…》 · English" cells to English-first
- editorial_histories.xlsx: normalize the one Chinese journal name to match

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/xlsx/editorial_histories.xlsx
+++ b/data/xlsx/editorial_histories.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Editorial Histories" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes &amp; Caveats" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Editorial Histories" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Notes &amp; Caveats" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Editorial Histories'!$A$1:$H$213</definedName>
@@ -8623,7 +8623,7 @@
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>Music Research / Yinyue Yanjiu (音乐研究)</t>
+          <t>Music Research (音乐研究)</t>
         </is>
       </c>
       <c r="B213" s="2" t="inlineStr">
@@ -8694,7 +8694,6 @@
           <t>atmimusic.com/jatmi-editorial-board-2</t>
         </is>
       </c>
-      <c r="H214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -8732,7 +8731,6 @@
           <t>atmimusic.com/jatmi-editorial-board-2</t>
         </is>
       </c>
-      <c r="H215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -8770,7 +8768,6 @@
           <t>symposium.music.org</t>
         </is>
       </c>
-      <c r="H216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -8808,7 +8805,6 @@
           <t>CMS archival bios</t>
         </is>
       </c>
-      <c r="H217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -8846,7 +8842,6 @@
           <t>symposium.music.org/40</t>
         </is>
       </c>
-      <c r="H218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -8884,7 +8879,6 @@
           <t>symposium.music.org/general-editor</t>
         </is>
       </c>
-      <c r="H219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -8922,7 +8916,6 @@
           <t>symposium.music.org/editors</t>
         </is>
       </c>
-      <c r="H220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -8960,7 +8953,6 @@
           <t>symposium.music.org/editors</t>
         </is>
       </c>
-      <c r="H221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -8998,7 +8990,6 @@
           <t>symposium.music.org/editors</t>
         </is>
       </c>
-      <c r="H222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -9036,7 +9027,6 @@
           <t>symposium.music.org/editors</t>
         </is>
       </c>
-      <c r="H223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -9074,7 +9064,6 @@
           <t>symposium.music.org/editors</t>
         </is>
       </c>
-      <c r="H224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -9112,7 +9101,6 @@
           <t>symposium.music.org/editors</t>
         </is>
       </c>
-      <c r="H225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -9150,7 +9138,6 @@
           <t>Update front matter (2004-05)</t>
         </is>
       </c>
-      <c r="H226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -9188,7 +9175,6 @@
           <t>nafme.org — interview with past editor</t>
         </is>
       </c>
-      <c r="H227" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H213"/>

</xml_diff>

<commit_message>
Sync updated editorial data; normalize Chinese names to English (简体)
Regenerated from the updated private masters via sync_public_data.py:
- editorial_histories.xlsx: latest editor records; Chinese journal names now
  show "English (简体)" instead of English/Pinyin (fixes the pinyin shown for
  China Music Education)
- journal_indexing.xlsx: Chinese journals English-first with simplified chars;
  removed the duplicate Music Research row

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/xlsx/editorial_histories.xlsx
+++ b/data/xlsx/editorial_histories.xlsx
@@ -8547,7 +8547,7 @@
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>China Music Education / Zhongguo Yinyue Jiaoyu</t>
+          <t>China Music Education (中国音乐教育)</t>
         </is>
       </c>
       <c r="B211" s="2" t="inlineStr">
@@ -8694,6 +8694,7 @@
           <t>atmimusic.com/jatmi-editorial-board-2</t>
         </is>
       </c>
+      <c r="H214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -8731,6 +8732,7 @@
           <t>atmimusic.com/jatmi-editorial-board-2</t>
         </is>
       </c>
+      <c r="H215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -8768,6 +8770,7 @@
           <t>symposium.music.org</t>
         </is>
       </c>
+      <c r="H216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -8805,6 +8808,7 @@
           <t>CMS archival bios</t>
         </is>
       </c>
+      <c r="H217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -8842,6 +8846,7 @@
           <t>symposium.music.org/40</t>
         </is>
       </c>
+      <c r="H218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -8879,6 +8884,7 @@
           <t>symposium.music.org/general-editor</t>
         </is>
       </c>
+      <c r="H219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -8916,6 +8922,7 @@
           <t>symposium.music.org/editors</t>
         </is>
       </c>
+      <c r="H220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -8953,6 +8960,7 @@
           <t>symposium.music.org/editors</t>
         </is>
       </c>
+      <c r="H221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -8990,6 +8998,7 @@
           <t>symposium.music.org/editors</t>
         </is>
       </c>
+      <c r="H222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -9027,6 +9036,7 @@
           <t>symposium.music.org/editors</t>
         </is>
       </c>
+      <c r="H223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -9064,6 +9074,7 @@
           <t>symposium.music.org/editors</t>
         </is>
       </c>
+      <c r="H224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -9101,6 +9112,7 @@
           <t>symposium.music.org/editors</t>
         </is>
       </c>
+      <c r="H225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -9138,6 +9150,7 @@
           <t>Update front matter (2004-05)</t>
         </is>
       </c>
+      <c r="H226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -9175,6 +9188,7 @@
           <t>nafme.org — interview with past editor</t>
         </is>
       </c>
+      <c r="H227" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H213"/>

</xml_diff>